<commit_message>
docs(query): service query set = 500 eval-only queries; plan synthetic training data
B 100->150, C 80->130 so B/C/A each get 100+ test queries. Human-written
queries are eval-only (dev 25% / test 75% per bundle); training data comes
from corpus-based generation (rules for names, LLM for intent/scenario,
cross-encoder filtering), documented in docs/SERVICE_QUERYSET.md section 4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/query/service_queryset_v1.xlsx
+++ b/data/query/service_queryset_v1.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -500,152 +500,164 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>용도</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>이 쿼리는 평가 전용(dev 25% / test 75%)이다. 학습에 쓰지 않는다.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>묶음 A</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>업종 확장 — 목표 150개</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>묶음 B</t>
+          <t>묶음 A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>상호명·브랜드 — 목표 100개</t>
+          <t>업종 확장 — 목표 150개</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>묶음 C</t>
+          <t>묶음 B</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>상품·상황 — 목표 80개</t>
+          <t>상호명·브랜드 — 목표 150개</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>묶음 D</t>
+          <t>묶음 C</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>지역+업종 — 목표 50개</t>
+          <t>상품·상황 — 목표 130개</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>묶음 D</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>지역+업종 — 목표 50개</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>묶음 E</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>결과 없음 — 목표 20개</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>A 업종 확장</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>A_업종후보에서 업종을 골라 4~5개씩. 유형 열에 T1 정확표기/T2 동의어/T3 개념확장/T4 구어·문장/T5 서비스.</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B 상호명</t>
+          <t>A 업종 확장</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>B_가맹점표본(S번호) 또는 B_체인목록(CH번호)을 보고 그 가게를 찾을 때 칠 말. 전체 이름, 일부, 브랜드만, 다른 표기(BBQ↔비비큐) 등. 의도 열에 찾는 상호.</t>
+          <t>A_업종후보에서 업종을 골라 4~5개씩. 유형 열에 T1 정확표기/T2 동의어/T3 개념확장/T4 구어·문장/T5 서비스.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C 상황</t>
+          <t>B 상호명</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C_상황카드(C번호)를 보고 1~3개. 의도 열에는 쓴 뒤에 '어떤 가게를 기대했는지'를 적는다.</t>
+          <t>B_가맹점표본(S번호) 또는 B_체인목록(CH번호)을 보고 그 가게를 찾을 때 칠 말. 전체 이름, 일부, 브랜드만, 다른 표기(BBQ↔비비큐) 등. 의도 열에 찾는 상호.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>D 지역+업종</t>
+          <t>C 상황</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>D_시장표본(M번호)의 지역·시장명 + 업종. 지역표현 열에 질의 속 지역 말, 가정위치ID에 M번호.</t>
+          <t>C_상황카드(C번호)를 보고 1~3개. 의도 열에는 쓴 뒤에 '어떤 가게를 기대했는지'를 적는다.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E 결과 없음</t>
+          <t>D 지역+업종</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>E_결과없음후보에서 '사용 가능'인 것 또는 직접 생각한 것. 온누리 가맹점이 아닐 법한 대상.</t>
+          <t>D_시장표본(M번호)의 지역·시장명 + 업종. 지역표현 열에 질의 속 지역 말, 가정위치ID에 M번호.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>가정위치ID</t>
+          <t>E 결과 없음</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>검색한 사람이 있다고 가정하는 위치(M번호). B는 비우면 표본 가맹점 위치. A·C·E는 비우면 나중에 자동 배정.</t>
+          <t>E_결과없음후보에서 '사용 가능'인 것 또는 직접 생각한 것. 온누리 가맹점이 아닐 법한 대상.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>가정위치ID</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>검색한 사람이 있다고 가정하는 위치(M번호). B는 비우면 표본 가맹점 위치. A·C·E는 비우면 나중에 자동 배정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>판정</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>사람은 업종·상호 관련성만 판정. 지역 일치는 주소·좌표로 자동 계산한다.</t>
         </is>

</xml_diff>